<commit_message>
pb with Date in NPOI lib
</commit_message>
<xml_diff>
--- a/2-Tests/Lexerow.Core.Tests/12-ExcelProcessorFiles/SetCellDate.xlsx
+++ b/2-Tests/Lexerow.Core.Tests/12-ExcelProcessorFiles/SetCellDate.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/a990f455bb745add/ProjetsDev/10-Pierlam/Lexerow/Dev/Lexerow/2-Tests/Lexerow.Core.Tests/12-ExcelProcessorFiles/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="50" documentId="11_2B8C63A238C272CACCFC3B895DC533011B7D74F5" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A612D2B1-B9B5-48EA-AAB2-3CF2DF4FD19D}"/>
+  <xr:revisionPtr revIDLastSave="71" documentId="11_2B8C63A238C272CACCFC3B895DC533011B7D74F5" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B3087429-ECD5-4B9D-97E3-2AAB2E29923A}"/>
   <bookViews>
-    <workbookView xWindow="9240" yWindow="8100" windowWidth="16515" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="13005" yWindow="1755" windowWidth="11610" windowHeight="10800" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
   <si>
     <t>null</t>
   </si>
@@ -75,13 +75,25 @@
   </si>
   <si>
     <t>formula</t>
+  </si>
+  <si>
+    <t>datetime</t>
+  </si>
+  <si>
+    <t>time</t>
+  </si>
+  <si>
+    <t>type</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd;@"/>
+  </numFmts>
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -96,8 +108,16 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -119,6 +139,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="3" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.79998168889431442"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -150,13 +176,19 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="14" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="14" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="14" fontId="1" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="22" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="21" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -441,19 +473,22 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C10"/>
+  <dimension ref="A1:C12"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="19.140625" customWidth="1"/>
-    <col min="2" max="2" width="15.5703125" customWidth="1"/>
+    <col min="2" max="2" width="19.7109375" customWidth="1"/>
     <col min="3" max="3" width="16.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="B1" t="s">
+      <c r="A1" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="B1" s="6" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="6" t="s">
         <v>8</v>
       </c>
     </row>
@@ -481,6 +516,9 @@
       <c r="B4" t="s">
         <v>4</v>
       </c>
+      <c r="C4" s="7">
+        <v>41595</v>
+      </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
@@ -516,7 +554,9 @@
       <c r="B8" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="C8" s="3"/>
+      <c r="C8" s="8">
+        <v>32043</v>
+      </c>
     </row>
     <row r="9" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
@@ -525,7 +565,9 @@
       <c r="B9" s="4">
         <v>23</v>
       </c>
-      <c r="C9" s="4"/>
+      <c r="C9" s="9">
+        <v>41333</v>
+      </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
@@ -535,8 +577,34 @@
         <f>B5+B6</f>
         <v>46.56</v>
       </c>
+      <c r="C10" s="2">
+        <v>43792</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>13</v>
+      </c>
+      <c r="B11" s="10">
+        <v>41012.479687500003</v>
+      </c>
+      <c r="C11" s="2">
+        <v>43329</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>14</v>
+      </c>
+      <c r="B12" s="11">
+        <v>0.52424768518518516</v>
+      </c>
+      <c r="C12" s="2">
+        <v>42201</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="4294967293" verticalDpi="0" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>